<commit_message>
guild hq testable checkpoint
</commit_message>
<xml_diff>
--- a/SkyreaderGuild/LangMod/EN/SourceCard.xlsx
+++ b/SkyreaderGuild/LangMod/EN/SourceCard.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="403">
   <si>
     <t>id</t>
   </si>
@@ -906,6 +906,330 @@
   </si>
   <si>
     <t>A shimmering gateway to an astral rift.</t>
+  </si>
+  <si>
+    <t>srg_aurora_lamp</t>
+  </si>
+  <si>
+    <t>オーロラランプ</t>
+  </si>
+  <si>
+    <t>aurora lamp</t>
+  </si>
+  <si>
+    <t>light</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/1,glass/2</t>
+  </si>
+  <si>
+    <t>Torch</t>
+  </si>
+  <si>
+    <t>candle_small</t>
+  </si>
+  <si>
+    <t>tourism</t>
+  </si>
+  <si>
+    <t>A softly glowing lamp that flickers with aurora-like light. Fragments of meteorite refract starlight through the glass.</t>
+  </si>
+  <si>
+    <t>srg_constellation_rug</t>
+  </si>
+  <si>
+    <t>星座のラグ</t>
+  </si>
+  <si>
+    <t>constellation rug</t>
+  </si>
+  <si>
+    <t>deco</t>
+  </si>
+  <si>
+    <t>@obj flat</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/1,texture/3</t>
+  </si>
+  <si>
+    <t>wool</t>
+  </si>
+  <si>
+    <t>A woven rug depicting star patterns. The constellation lines seem to shimmer faintly.</t>
+  </si>
+  <si>
+    <t>srg_starfall_table</t>
+  </si>
+  <si>
+    <t>星降りのテーブル</t>
+  </si>
+  <si>
+    <t>starfall table</t>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/2,plank/4</t>
+  </si>
+  <si>
+    <t>A sturdy table inlaid with fragments of meteorite. The surface catches light in strange ways.</t>
+  </si>
+  <si>
+    <t>srg_lunar_armchair</t>
+  </si>
+  <si>
+    <t>月のアームチェア</t>
+  </si>
+  <si>
+    <t>lunar armchair</t>
+  </si>
+  <si>
+    <t>chair</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/2,texture/3,stick/2</t>
+  </si>
+  <si>
+    <t>Chair</t>
+  </si>
+  <si>
+    <t>A plush armchair upholstered with star-patterned fabric. The crescent moon motif on the backrest glows faintly.</t>
+  </si>
+  <si>
+    <t>srg_celestial_globe</t>
+  </si>
+  <si>
+    <t>天球儀</t>
+  </si>
+  <si>
+    <t>celestial globe</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/2,glass/3</t>
+  </si>
+  <si>
+    <t>A glass sphere on a brass stand showing constellations. The star-lines glow with captured starlight.</t>
+  </si>
+  <si>
+    <t>srg_zodiac_dresser</t>
+  </si>
+  <si>
+    <t>星座のドレッサー</t>
+  </si>
+  <si>
+    <t>zodiac dresser</t>
+  </si>
+  <si>
+    <t>container</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/3,plank/6,bolt/2</t>
+  </si>
+  <si>
+    <t>Container,5,4,crate</t>
+  </si>
+  <si>
+    <t>Storeroom,Stockroom</t>
+  </si>
+  <si>
+    <t>A dresser carved with zodiac symbols. Each drawer is perfectly balanced for storing stargazing instruments.</t>
+  </si>
+  <si>
+    <t>srg_cosmic_mirror</t>
+  </si>
+  <si>
+    <t>宇宙の鏡</t>
+  </si>
+  <si>
+    <t>cosmic mirror</t>
+  </si>
+  <si>
+    <t>_furniture</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/3,glass/6,plank/2</t>
+  </si>
+  <si>
+    <t>Mirror</t>
+  </si>
+  <si>
+    <t>A standing mirror framed in meteorite-laced silver. The reflection ripples with astral distortion.</t>
+  </si>
+  <si>
+    <t>srg_planisphere_cabinet</t>
+  </si>
+  <si>
+    <t>天球キャビネット</t>
+  </si>
+  <si>
+    <t>planisphere cabinet</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/3,plank/8,glass/2</t>
+  </si>
+  <si>
+    <t>BookShelf</t>
+  </si>
+  <si>
+    <t>A tall cabinet displaying star charts behind glass doors. The planisphere mechanism rotates slowly.</t>
+  </si>
+  <si>
+    <t>srg_stardust_bed</t>
+  </si>
+  <si>
+    <t>星塵のベッド</t>
+  </si>
+  <si>
+    <t>stardust bed</t>
+  </si>
+  <si>
+    <t>bed</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/4,texture/6,plank/4</t>
+  </si>
+  <si>
+    <t>cotton</t>
+  </si>
+  <si>
+    <t>Bed,2</t>
+  </si>
+  <si>
+    <t>Bedroom</t>
+  </si>
+  <si>
+    <t>A bed woven with stardust fibers. Sleepers report dreams of distant nebulae.</t>
+  </si>
+  <si>
+    <t>srg_astral_chandelier</t>
+  </si>
+  <si>
+    <t>星霊のシャンデリア</t>
+  </si>
+  <si>
+    <t>astral chandelier</t>
+  </si>
+  <si>
+    <t>mount</t>
+  </si>
+  <si>
+    <t>ObjFloat</t>
+  </si>
+  <si>
+    <t>@obj ceil</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/4,ingot/4,gem/2</t>
+  </si>
+  <si>
+    <t>A chandelier of crystallized starlight suspended from the ceiling. Its light dances like captured constellations.</t>
+  </si>
+  <si>
+    <t>srg_meteorite_statue</t>
+  </si>
+  <si>
+    <t>隕石の彫像</t>
+  </si>
+  <si>
+    <t>meteorite statue</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/5,cutstone/8,ingot/4</t>
+  </si>
+  <si>
+    <t>fireproof/1,acidproof/1</t>
+  </si>
+  <si>
+    <t>A towering statue carved from meteorite stone. Cosmic cracks glow with trapped starlight.</t>
+  </si>
+  <si>
+    <t>srg_eclipse_hearth</t>
+  </si>
+  <si>
+    <t>蝕のかまど</t>
+  </si>
+  <si>
+    <t>eclipse hearth</t>
+  </si>
+  <si>
+    <t>srg_meteorite_source/6,cutstone/10,brick/6,ingot/4</t>
+  </si>
+  <si>
+    <t>Hearth,cooking</t>
+  </si>
+  <si>
+    <t>fireplace</t>
+  </si>
+  <si>
+    <t>amb_fire</t>
+  </si>
+  <si>
+    <t>Kitchen,Dining Room</t>
+  </si>
+  <si>
+    <t>A grand hearth carved with eclipse motifs. The flames burn with starfire and can cook any meal.</t>
+  </si>
+  <si>
+    <t>srg_guild_entrance</t>
+  </si>
+  <si>
+    <t>Skyreader Observatory gateway</t>
+  </si>
+  <si>
+    <t>mech</t>
+  </si>
+  <si>
+    <t>furniture_mech</t>
+  </si>
+  <si>
+    <t>obj tall</t>
+  </si>
+  <si>
+    <t>ether</t>
+  </si>
+  <si>
+    <t>SkyreaderGuildEntrance,srg_guild_hq</t>
+  </si>
+  <si>
+    <t>noWish,noShop</t>
+  </si>
+  <si>
+    <t>Portal Room</t>
+  </si>
+  <si>
+    <t>A shimmering astral gate leading to the Skyreader Observatory.</t>
+  </si>
+  <si>
+    <t>srg_guild_exit</t>
+  </si>
+  <si>
+    <t>Derphy gateway</t>
+  </si>
+  <si>
+    <t>SkyreaderGuildExit</t>
+  </si>
+  <si>
+    <t>A shimmering astral gate leading back to Derphy.</t>
+  </si>
+  <si>
+    <t>srg_nexus_core</t>
+  </si>
+  <si>
+    <t>巨大なる隕石の核</t>
+  </si>
+  <si>
+    <t>nexus meteor core</t>
+  </si>
+  <si>
+    <t>@obj_LV</t>
+  </si>
+  <si>
+    <t>tourism,noShop</t>
+  </si>
+  <si>
+    <t>A colossal, perfectly preserved meteor core pulled from an astral rift. It hums with the terrifying song of deep space.</t>
   </si>
 </sst>
 </file>
@@ -2736,7 +3060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ17"/>
+  <dimension ref="A1:AZ32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="7.42578125" defaultRowHeight="16.5"/>
   <cols>
     <col width="14.140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -3928,6 +4252,804 @@
         <v>294</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>295</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>296</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>297</v>
+      </c>
+      <c r="I18" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="M18" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="N18" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U18" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V18" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W18" s="0" t="s">
+        <v>299</v>
+      </c>
+      <c r="Y18" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA18" s="0" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AB18" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC18" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="0" t="n">
+        <v>800</v>
+      </c>
+      <c r="AH18" s="0" t="s">
+        <v>300</v>
+      </c>
+      <c r="AO18" s="0" t="s">
+        <v>301</v>
+      </c>
+      <c r="AT18" s="0" t="s">
+        <v>302</v>
+      </c>
+      <c r="AZ18" s="0" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>304</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>305</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>306</v>
+      </c>
+      <c r="I19" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="M19" s="0" t="s">
+        <v>308</v>
+      </c>
+      <c r="N19" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U19" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V19" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W19" s="0" t="s">
+        <v>309</v>
+      </c>
+      <c r="Y19" s="0" t="s">
+        <v>310</v>
+      </c>
+      <c r="AA19" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="AB19" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="0" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AZ19" s="0" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
+        <v>312</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>313</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>314</v>
+      </c>
+      <c r="I20" s="0" t="s">
+        <v>315</v>
+      </c>
+      <c r="M20" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N20" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U20" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V20" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W20" s="0" t="s">
+        <v>316</v>
+      </c>
+      <c r="Y20" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA20" s="0" t="n">
+        <v>3200</v>
+      </c>
+      <c r="AB20" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="0" t="n">
+        <v>6000</v>
+      </c>
+      <c r="AZ20" s="0" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="s">
+        <v>318</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>319</v>
+      </c>
+      <c r="F21" s="0" t="s">
+        <v>320</v>
+      </c>
+      <c r="I21" s="0" t="s">
+        <v>321</v>
+      </c>
+      <c r="M21" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N21" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U21" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V21" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W21" s="0" t="s">
+        <v>322</v>
+      </c>
+      <c r="Y21" s="0" t="s">
+        <v>310</v>
+      </c>
+      <c r="AA21" s="0" t="n">
+        <v>3600</v>
+      </c>
+      <c r="AB21" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="0" t="n">
+        <v>4500</v>
+      </c>
+      <c r="AH21" s="0" t="s">
+        <v>323</v>
+      </c>
+      <c r="AZ21" s="0" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
+        <v>325</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>326</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>327</v>
+      </c>
+      <c r="I22" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="M22" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="N22" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U22" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V22" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W22" s="0" t="s">
+        <v>328</v>
+      </c>
+      <c r="Y22" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA22" s="0" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB22" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AT22" s="0" t="s">
+        <v>302</v>
+      </c>
+      <c r="AZ22" s="0" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="s">
+        <v>330</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>331</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>332</v>
+      </c>
+      <c r="I23" s="0" t="s">
+        <v>333</v>
+      </c>
+      <c r="M23" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N23" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U23" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V23" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W23" s="0" t="s">
+        <v>334</v>
+      </c>
+      <c r="Y23" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA23" s="0" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AB23" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="AC23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="0" t="n">
+        <v>12000</v>
+      </c>
+      <c r="AH23" s="0" t="s">
+        <v>335</v>
+      </c>
+      <c r="AX23" s="0" t="s">
+        <v>336</v>
+      </c>
+      <c r="AZ23" s="0" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="s">
+        <v>338</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>339</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>340</v>
+      </c>
+      <c r="I24" s="0" t="s">
+        <v>341</v>
+      </c>
+      <c r="M24" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N24" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U24" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V24" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W24" s="0" t="s">
+        <v>342</v>
+      </c>
+      <c r="Y24" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA24" s="0" t="n">
+        <v>5500</v>
+      </c>
+      <c r="AB24" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" s="0" t="n">
+        <v>7000</v>
+      </c>
+      <c r="AH24" s="0" t="s">
+        <v>343</v>
+      </c>
+      <c r="AZ24" s="0" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>346</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>347</v>
+      </c>
+      <c r="I25" s="0" t="s">
+        <v>333</v>
+      </c>
+      <c r="L25" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M25" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N25" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U25" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V25" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W25" s="0" t="s">
+        <v>348</v>
+      </c>
+      <c r="Y25" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA25" s="0" t="n">
+        <v>6000</v>
+      </c>
+      <c r="AB25" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="0" t="n">
+        <v>15000</v>
+      </c>
+      <c r="AH25" s="0" t="s">
+        <v>349</v>
+      </c>
+      <c r="AZ25" s="0" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="s">
+        <v>351</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>352</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>353</v>
+      </c>
+      <c r="I26" s="0" t="s">
+        <v>354</v>
+      </c>
+      <c r="M26" s="0" t="s">
+        <v>308</v>
+      </c>
+      <c r="N26" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U26" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V26" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W26" s="0" t="s">
+        <v>355</v>
+      </c>
+      <c r="Y26" s="0" t="s">
+        <v>356</v>
+      </c>
+      <c r="AA26" s="0" t="n">
+        <v>8000</v>
+      </c>
+      <c r="AB26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="0" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AH26" s="0" t="s">
+        <v>357</v>
+      </c>
+      <c r="AX26" s="0" t="s">
+        <v>358</v>
+      </c>
+      <c r="AZ26" s="0" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="s">
+        <v>360</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>361</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>362</v>
+      </c>
+      <c r="I27" s="0" t="s">
+        <v>363</v>
+      </c>
+      <c r="L27" s="0" t="s">
+        <v>364</v>
+      </c>
+      <c r="M27" s="0" t="s">
+        <v>365</v>
+      </c>
+      <c r="N27" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U27" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V27" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W27" s="0" t="s">
+        <v>366</v>
+      </c>
+      <c r="Y27" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="AA27" s="0" t="n">
+        <v>9000</v>
+      </c>
+      <c r="AB27" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="AC27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="0" t="n">
+        <v>6000</v>
+      </c>
+      <c r="AH27" s="0" t="s">
+        <v>300</v>
+      </c>
+      <c r="AO27" s="0" t="s">
+        <v>301</v>
+      </c>
+      <c r="AT27" s="0" t="s">
+        <v>302</v>
+      </c>
+      <c r="AZ27" s="0" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="s">
+        <v>368</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>370</v>
+      </c>
+      <c r="I28" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="L28" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M28" s="0" t="s">
+        <v>290</v>
+      </c>
+      <c r="N28" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U28" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V28" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W28" s="0" t="s">
+        <v>371</v>
+      </c>
+      <c r="Y28" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="AA28" s="0" t="n">
+        <v>15000</v>
+      </c>
+      <c r="AB28" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="0" t="n">
+        <v>35000</v>
+      </c>
+      <c r="AI28" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="AT28" s="0" t="s">
+        <v>302</v>
+      </c>
+      <c r="AZ28" s="0" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="s">
+        <v>374</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="F29" s="0" t="s">
+        <v>376</v>
+      </c>
+      <c r="I29" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="M29" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N29" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="U29" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="V29" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="W29" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="Y29" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="AA29" s="0" t="n">
+        <v>20000</v>
+      </c>
+      <c r="AB29" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="AC29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="0" t="n">
+        <v>25000</v>
+      </c>
+      <c r="AH29" s="0" t="s">
+        <v>378</v>
+      </c>
+      <c r="AO29" s="0" t="s">
+        <v>379</v>
+      </c>
+      <c r="AP29" s="0" t="s">
+        <v>379</v>
+      </c>
+      <c r="AQ29" s="0" t="s">
+        <v>379</v>
+      </c>
+      <c r="AS29" s="0" t="s">
+        <v>380</v>
+      </c>
+      <c r="AX29" s="0" t="s">
+        <v>381</v>
+      </c>
+      <c r="AZ29" s="0" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="s">
+        <v>383</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>384</v>
+      </c>
+      <c r="I30" s="0" t="s">
+        <v>385</v>
+      </c>
+      <c r="J30" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="M30" s="0" t="s">
+        <v>387</v>
+      </c>
+      <c r="N30" s="0" t="n">
+        <v>751</v>
+      </c>
+      <c r="O30" s="0" t="n">
+        <v>752</v>
+      </c>
+      <c r="P30" s="0" t="s">
+        <v>291</v>
+      </c>
+      <c r="Y30" s="0" t="s">
+        <v>388</v>
+      </c>
+      <c r="AA30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF30" s="0" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AH30" s="0" t="s">
+        <v>389</v>
+      </c>
+      <c r="AT30" s="0" t="s">
+        <v>390</v>
+      </c>
+      <c r="AX30" s="0" t="s">
+        <v>391</v>
+      </c>
+      <c r="AZ30" s="0" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="s">
+        <v>393</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>394</v>
+      </c>
+      <c r="I31" s="0" t="s">
+        <v>385</v>
+      </c>
+      <c r="J31" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="M31" s="0" t="s">
+        <v>387</v>
+      </c>
+      <c r="N31" s="0" t="n">
+        <v>751</v>
+      </c>
+      <c r="O31" s="0" t="n">
+        <v>752</v>
+      </c>
+      <c r="P31" s="0" t="s">
+        <v>291</v>
+      </c>
+      <c r="Y31" s="0" t="s">
+        <v>388</v>
+      </c>
+      <c r="AA31" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC31" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF31" s="0" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AH31" s="0" t="s">
+        <v>395</v>
+      </c>
+      <c r="AT31" s="0" t="s">
+        <v>390</v>
+      </c>
+      <c r="AX31" s="0" t="s">
+        <v>391</v>
+      </c>
+      <c r="AZ31" s="0" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>398</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>399</v>
+      </c>
+      <c r="I32" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="L32" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M32" s="0" t="s">
+        <v>400</v>
+      </c>
+      <c r="N32" s="0" t="n">
+        <v>503</v>
+      </c>
+      <c r="Y32" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="AA32" s="0" t="n">
+        <v>50000</v>
+      </c>
+      <c r="AB32" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="AC32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" s="0" t="n">
+        <v>99999</v>
+      </c>
+      <c r="AI32" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="AT32" s="0" t="s">
+        <v>401</v>
+      </c>
+      <c r="AZ32" s="0" t="s">
+        <v>402</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:AZ3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
testable async features checkpoint
</commit_message>
<xml_diff>
--- a/SkyreaderGuild/LangMod/EN/SourceCard.xlsx
+++ b/SkyreaderGuild/LangMod/EN/SourceCard.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="431">
   <si>
     <t>id</t>
   </si>
@@ -1245,6 +1245,75 @@
   </si>
   <si>
     <t>A guild plaque covered with carefully updated rankings.</t>
+  </si>
+  <si>
+    <t>srg_constellation_board</t>
+  </si>
+  <si>
+    <t>constellation board</t>
+  </si>
+  <si>
+    <t>ConstellationBoard</t>
+  </si>
+  <si>
+    <t>Observatory</t>
+  </si>
+  <si>
+    <t>A board displaying the five patron constellations of the season. Each tells a different cosmic story.</t>
+  </si>
+  <si>
+    <t>srg_geometry_orrery</t>
+  </si>
+  <si>
+    <t>geometry orrery</t>
+  </si>
+  <si>
+    <t>bronze</t>
+  </si>
+  <si>
+    <t>GeometryOrrery</t>
+  </si>
+  <si>
+    <t>A mechanical device tracking the dominant geometry of astral rifts across all Skyreaders.</t>
+  </si>
+  <si>
+    <t>srg_comet_heatmap_table</t>
+  </si>
+  <si>
+    <t>astral contamination table</t>
+  </si>
+  <si>
+    <t>CometHeatmapTable</t>
+  </si>
+  <si>
+    <t>A table mapping astral contamination from meteor-touched townspeople and items.</t>
+  </si>
+  <si>
+    <t>srg_star_paper_shelf</t>
+  </si>
+  <si>
+    <t>star paper shelf</t>
+  </si>
+  <si>
+    <t>StarPaperShelf</t>
+  </si>
+  <si>
+    <t>Library</t>
+  </si>
+  <si>
+    <t>A shelf housing anonymous research notes submitted by Skyreaders across the world.</t>
+  </si>
+  <si>
+    <t>srg_star_paper_desk</t>
+  </si>
+  <si>
+    <t>star paper writing desk</t>
+  </si>
+  <si>
+    <t>StarPaperWritingDesk</t>
+  </si>
+  <si>
+    <t>A writing desk for composing star papers. The ink shimmers faintly.</t>
   </si>
 </sst>
 </file>
@@ -3075,7 +3144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ33"/>
+  <dimension ref="A1:AZ38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="7.42578125" defaultRowHeight="16.5"/>
   <cols>
     <col width="14.140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -5113,6 +5182,253 @@
         <v>407</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="0" t="s">
+        <v>408</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>409</v>
+      </c>
+      <c r="I34" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="L34" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M34" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N34" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="Y34" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA34" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AB34" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF34" s="0" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AH34" s="0" t="s">
+        <v>410</v>
+      </c>
+      <c r="AT34" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="AX34" s="0" t="s">
+        <v>411</v>
+      </c>
+      <c r="AZ34" s="0" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="s">
+        <v>413</v>
+      </c>
+      <c r="F35" s="0" t="s">
+        <v>414</v>
+      </c>
+      <c r="I35" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="L35" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M35" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N35" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="Y35" s="0" t="s">
+        <v>415</v>
+      </c>
+      <c r="AA35" s="0" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB35" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF35" s="0" t="n">
+        <v>8000</v>
+      </c>
+      <c r="AH35" s="0" t="s">
+        <v>416</v>
+      </c>
+      <c r="AT35" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="AX35" s="0" t="s">
+        <v>411</v>
+      </c>
+      <c r="AZ35" s="0" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="s">
+        <v>418</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>419</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="L36" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M36" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N36" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="Y36" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA36" s="0" t="n">
+        <v>2500</v>
+      </c>
+      <c r="AB36" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF36" s="0" t="n">
+        <v>6000</v>
+      </c>
+      <c r="AH36" s="0" t="s">
+        <v>420</v>
+      </c>
+      <c r="AT36" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="AX36" s="0" t="s">
+        <v>411</v>
+      </c>
+      <c r="AZ36" s="0" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="s">
+        <v>422</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>423</v>
+      </c>
+      <c r="I37" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="L37" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="M37" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N37" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="Y37" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA37" s="0" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AB37" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF37" s="0" t="n">
+        <v>7000</v>
+      </c>
+      <c r="AH37" s="0" t="s">
+        <v>424</v>
+      </c>
+      <c r="AT37" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="AX37" s="0" t="s">
+        <v>425</v>
+      </c>
+      <c r="AZ37" s="0" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="s">
+        <v>427</v>
+      </c>
+      <c r="F38" s="0" t="s">
+        <v>428</v>
+      </c>
+      <c r="I38" s="0" t="s">
+        <v>307</v>
+      </c>
+      <c r="M38" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="N38" s="0" t="n">
+        <v>1552</v>
+      </c>
+      <c r="Y38" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA38" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="AB38" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF38" s="0" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AH38" s="0" t="s">
+        <v>429</v>
+      </c>
+      <c r="AT38" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="AX38" s="0" t="s">
+        <v>425</v>
+      </c>
+      <c r="AZ38" s="0" t="s">
+        <v>430</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:AZ3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>